<commit_message>
Earn2Trade : campagne de fin septembre, SCANNED a 60 %
Offre portee a 60 % jusqu'au 30 septembre fin de journee heure du Centre
(1er octobre 05:00 UTC), portee universelle, checkout verifie. La
condition des trois mois et les prix de reset de la campagne sont dans
les couts.

Le coupon SCANNED est confirme par le panneau d'affiliation Earn2Trade :
c'est le coupon personnel de Sofiane, celui qui trace ses commissions.

Correctif generique : ficheAffichable masque desormais une offre dont la
date de fin est passee. Sans lui, une campagne de trois jours serait
restee affichee jusqu'a ce que quelqu'un modifie le tableur.

Deux fichiers SQL pour la mise en avant sur /compare : priority_tier a 1
pendant la campagne, et son retour le 1er octobre.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/firms/earn2trade.xlsx
+++ b/data/firms/earn2trade.xlsx
@@ -1374,7 +1374,7 @@
         </is>
       </c>
       <c r="B3" s="31" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="C3" s="30" t="n">
         <v>0.3</v>
@@ -1393,7 +1393,7 @@
       </c>
       <c r="B4" s="16" t="inlineStr">
         <is>
-          <t>non_confirmee</t>
+          <t>universelle_verifiee</t>
         </is>
       </c>
       <c r="C4" s="17" t="inlineStr">
@@ -1415,7 +1415,7 @@
       </c>
       <c r="B5" s="16" t="inlineStr">
         <is>
-          <t>non</t>
+          <t>oui</t>
         </is>
       </c>
       <c r="C5" s="17" t="inlineStr">
@@ -1471,7 +1471,11 @@
           <t>expire_le</t>
         </is>
       </c>
-      <c r="B8" s="32" t="n"/>
+      <c r="B8" s="32" t="inlineStr">
+        <is>
+          <t>2026-10-01T05:00:00+00:00</t>
+        </is>
+      </c>
       <c r="C8" s="33" t="inlineStr">
         <is>
           <t>(vide — date de fin inconnue)</t>
@@ -2397,10 +2401,24 @@
       <c r="E5" s="16" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="23" t="n"/>
-      <c r="B6" s="16" t="n"/>
-      <c r="C6" s="16" t="n"/>
-      <c r="D6" s="16" t="n"/>
+      <c r="A6" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>End of September offer</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>-60% for 3 months</t>
+        </is>
+      </c>
+      <c r="D6" s="16" t="inlineStr">
+        <is>
+          <t>Until 30 September, end of day Central Time, code SCANNED takes 60% off instead of 50%, on the first three monthly billings. Resets are cheaper over the same three months: $55 on TCP25, $65 on TCP50, $60 on GAU50. After that, the code returns to 50% on every billing.</t>
+        </is>
+      </c>
       <c r="E6" s="16" t="n"/>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
Earn2Trade : la reinitialisation offerte apparait sur la fiche
Eva Saint-Arroman (affiliation Earn2Trade, 29/09) : la promo, c'est deux
choses, et la seconde manquait — une reinitialisation offerte avec chaque
evaluation. Verifie sur leur propre banniere le 29/09 : « Ends Sep 30: 60%
OFF + a FREE Reset With Every Evaluation ».

- Accroche : « Plus a free reset with every evaluation — until Sep 30. »
- Ligne « End of September offer » des couts : montant et note le disent.
- La fiche affiche desormais l'accroche sous le pourcentage ; elle ne vivait
  que dans le bandeau. Vide dans le tableur, rien ne s'affiche : la regle
  vaut pour toutes les firmes.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/firms/earn2trade.xlsx
+++ b/data/firms/earn2trade.xlsx
@@ -1513,7 +1513,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>60% off + a free reset with every evaluation. Ends Sep 30.</t>
+          <t>Plus a free reset with every evaluation — until Sep 30.</t>
         </is>
       </c>
       <c r="D10" s="15" t="inlineStr">
@@ -2456,12 +2456,12 @@
       </c>
       <c r="C6" s="16" t="inlineStr">
         <is>
-          <t>-60% for 3 months</t>
+          <t>-60% + free reset</t>
         </is>
       </c>
       <c r="D6" s="16" t="inlineStr">
         <is>
-          <t>Until 30 September, end of day Central Time, code SCANNED takes 60% off instead of 50%, on the first three monthly billings. Resets are cheaper over the same three months: $55 on TCP25, $65 on TCP50, $60 on GAU50. After that, the code returns to 50% on every billing.</t>
+          <t>Until 30 September, end of day Central Time, code SCANNED takes 60% off instead of 50%, on the first three monthly billings, and every evaluation comes with a free reset. Reset prices over the same three months: $55 on TCP25, $65 on TCP50, $60 on GAU50. After that, the code returns to 50% on every billing.</t>
         </is>
       </c>
       <c r="E6" s="16" t="n"/>

</xml_diff>

<commit_message>
Earn2Trade : le reset offert s'acquiert a l'achat, pas au renouvellement
Precision de Sofiane (29/09) : acheter une evaluation avant la fin de la promo
donne une reinitialisation offerte — une seconde tentative sans repayer.
« Avec chaque evaluation » laissait croire a un avantage recurrent.

- Accroche : « One free reset comes with it: a second attempt, nothing more to
  pay. Until Sep 30. »
- Couts : « -60% + 1 free reset », et la note relie enfin les deux phrases —
  le premier reset est offert, les suivants coutent $55 / $65 / $60.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/firms/earn2trade.xlsx
+++ b/data/firms/earn2trade.xlsx
@@ -1513,7 +1513,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Plus a free reset with every evaluation — until Sep 30.</t>
+          <t>One free reset comes with it: a second attempt, nothing more to pay. Until Sep 30.</t>
         </is>
       </c>
       <c r="D10" s="15" t="inlineStr">
@@ -2456,12 +2456,12 @@
       </c>
       <c r="C6" s="16" t="inlineStr">
         <is>
-          <t>-60% + free reset</t>
+          <t>-60% + 1 free reset</t>
         </is>
       </c>
       <c r="D6" s="16" t="inlineStr">
         <is>
-          <t>Until 30 September, end of day Central Time, code SCANNED takes 60% off instead of 50%, on the first three monthly billings, and every evaluation comes with a free reset. Reset prices over the same three months: $55 on TCP25, $65 on TCP50, $60 on GAU50. After that, the code returns to 50% on every billing.</t>
+          <t>Until 30 September, end of day Central Time, code SCANNED takes 60% off instead of 50% on the first three monthly billings. Every evaluation bought before the deadline also comes with one free reset: fail it, restart it, nothing more to pay. Any further reset costs $55 on TCP25, $65 on TCP50, $60 on GAU50 over the same three months. After that, the code returns to 50% on every billing.</t>
         </is>
       </c>
       <c r="E6" s="16" t="n"/>

</xml_diff>

<commit_message>
Earn2Trade : chaque plan ouvre SON checkout, code applique
Le configurateur envoyait le visiteur sur le plan d'entree quoi qu'il
choisisse : la colonne lien_plan etait vide, donc /api/go n'avait aucun plan a
resoudre et retombait sur le sauvetage coupon, c'est-a-dire le moins cher.

Les sept plans portent desormais leur identifiant en base — verifie ligne a
ligne, meme programme, meme taille, meme prix. Les sept sorties ont ete
testees : TCP25/50/100 et GAU50/100/150/200 ouvrent leur propre checkout,
« Coupon: scanned » applique, avec l'identifiant d'affiliation propre au
programme (a_bid different entre Trader Career Path et Gauntlet Mini).
Verifie jusqu'au panier sur GAU200 : 550 $ - 330 $ = 220 $/mois.

Pour que la panne ne revienne pas en silence, la generation avertit desormais
quand une fiche annonce une offre testee au checkout mais laisse des plans
sans lien_plan. Elle signale deja Blueberry Funded.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/firms/earn2trade.xlsx
+++ b/data/firms/earn2trade.xlsx
@@ -7059,6 +7059,11 @@
         <f>IF(A3="","",IF(COUNTIF(Programmes!$A$3:$A$60,A3)=0,"programme inconnu",IF(K3=0,"aucune phase","ok")))</f>
         <v/>
       </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>earn2trade-tcp25</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="16" t="inlineStr">
@@ -7099,6 +7104,11 @@
         <f>IF(A4="","",IF(COUNTIF(Programmes!$A$3:$A$60,A4)=0,"programme inconnu",IF(K4=0,"aucune phase","ok")))</f>
         <v/>
       </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>earn2trade-tcp50</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="16" t="inlineStr">
@@ -7140,6 +7150,11 @@
       <c r="L5" s="28">
         <f>IF(A5="","",IF(COUNTIF(Programmes!$A$3:$A$60,A5)=0,"programme inconnu",IF(K5=0,"aucune phase","ok")))</f>
         <v/>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>earn2trade-tcp100</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -7181,6 +7196,11 @@
         <f>IF(A6="","",IF(COUNTIF(Programmes!$A$3:$A$60,A6)=0,"programme inconnu",IF(K6=0,"aucune phase","ok")))</f>
         <v/>
       </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>earn2trade-gm50</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="16" t="inlineStr">
@@ -7223,6 +7243,11 @@
         <f>IF(A7="","",IF(COUNTIF(Programmes!$A$3:$A$60,A7)=0,"programme inconnu",IF(K7=0,"aucune phase","ok")))</f>
         <v/>
       </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>earn2trade-gm100</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="16" t="inlineStr">
@@ -7265,6 +7290,11 @@
         <f>IF(A8="","",IF(COUNTIF(Programmes!$A$3:$A$60,A8)=0,"programme inconnu",IF(K8=0,"aucune phase","ok")))</f>
         <v/>
       </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>earn2trade-gm150</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="16" t="inlineStr">
@@ -7306,6 +7336,11 @@
       <c r="L9" s="28">
         <f>IF(A9="","",IF(COUNTIF(Programmes!$A$3:$A$60,A9)=0,"programme inconnu",IF(K9=0,"aucune phase","ok")))</f>
         <v/>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>earn2trade-gm200</t>
+        </is>
       </c>
     </row>
     <row r="10">

</xml_diff>

<commit_message>
Earn2Trade : les 10 ans remplacent la campagne de septembre
Courriel de l'equipe affiliation du 1er octobre. Seules les deux offres que ce
courriel declare publiques sont publiees :
  - pack anniversaire, jusqu'au 10 : trois evaluations TCP25 et trois resets
    pour 165 $, soit 27,50 $ la tentative, dans la limite des stocks ;
  - offre generale, du 2 au 18 : 50 % sur toute evaluation TCP ou GAU, et 50 %
    sur les resets pendant 90 jours.

Le calendrier des dix offres quotidiennes est sous embargo a leur demande : il
n'est ni dans la fiche, ni dans ce depot, ni nulle part sur le site.

Ni taux de campagne ni pastille : le code reste a 50 % avant, pendant et
apres, donc un compte a rebours promettrait une fin qui n'existe pas, et une
pastille decalerait de nouveau la rangee de /compare. L'accroche porte
l'anniversaire, les deux lignes de couts portent le detail.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/firms/earn2trade.xlsx
+++ b/data/firms/earn2trade.xlsx
@@ -1513,7 +1513,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Flash offer — free reset included. Until Sep 30 only.</t>
+          <t>Earn2Trade turns 10: anniversary offers until 18 October.</t>
         </is>
       </c>
       <c r="D10" s="15" t="inlineStr">
@@ -1528,9 +1528,6 @@
           <t>remise_campagne</t>
         </is>
       </c>
-      <c r="B11" t="n">
-        <v>0.6</v>
-      </c>
       <c r="D11" s="15" t="inlineStr">
         <is>
           <t>Taux d'une campagne a duree limitee, en %. Il remplace « remise » jusqu'a « campagne_fin », puis la fiche revient a « remise ».</t>
@@ -1543,11 +1540,6 @@
           <t>campagne_fin</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>2026-10-01T05:00:00+00:00</t>
-        </is>
-      </c>
       <c r="D12" s="15" t="inlineStr">
         <is>
           <t>Fin de la campagne, date et heure ISO. Passee, le taux de campagne et l'accroche disparaissent, l'offre permanente reste.</t>
@@ -1558,11 +1550,6 @@
       <c r="A13" s="15" t="inlineStr">
         <is>
           <t>bonus</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>+1 free reset</t>
         </is>
       </c>
       <c r="D13" s="15" t="inlineStr">
@@ -2468,26 +2455,40 @@
       </c>
       <c r="B6" s="16" t="inlineStr">
         <is>
-          <t>End of September offer</t>
+          <t>Anniversary pack</t>
         </is>
       </c>
       <c r="C6" s="16" t="inlineStr">
         <is>
-          <t>-60% + 1 free reset</t>
+          <t>$165 for three</t>
         </is>
       </c>
       <c r="D6" s="16" t="inlineStr">
         <is>
-          <t>Until 30 September, end of day Central Time, code SCANNED takes 60% off instead of 50% on the first three monthly billings. Every evaluation bought before the deadline also comes with one free reset: fail it, restart it, nothing more to pay. Any further reset costs $55 on TCP25, $65 on TCP50, $60 on GAU50 over the same three months. After that, the code returns to 50% on every billing.</t>
+          <t>Until 10 October, three TCP25 evaluations and three resets for a single $165 payment — $27.50 per attempt. While stocks last.</t>
         </is>
       </c>
       <c r="E6" s="16" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="23" t="n"/>
-      <c r="B7" s="16" t="n"/>
-      <c r="C7" s="16" t="n"/>
-      <c r="D7" s="16" t="n"/>
+      <c r="A7" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Anniversary offer</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>-50% until 18 Oct</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>From 2 to 18 October, 50% off any Trader Career Path or Gauntlet Mini evaluation, and 50% off resets for the first 90 days.</t>
+        </is>
+      </c>
       <c r="E7" s="16" t="n"/>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Earn2Trade : le plan mis en avant passe au 50 K
Information de Sofiane (06/10) : c'est le compte a 50 000 $ qui se vend le
mieux. Leur site, lui, marque « Most Popular » sur le programme Trader Career
Path, pas sur une taille — j'ai donc retenu le TCP 50 K, soit ce programme a
cette taille, et non le Gauntlet Mini 50 K.

La carte du haut de fiche affiche desormais 190 $ au lieu de 150, et son
bouton ouvre le checkout du TCP50 (lien earn2trade-tcp50) au lieu du TCP25.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/firms/earn2trade.xlsx
+++ b/data/firms/earn2trade.xlsx
@@ -7444,11 +7444,7 @@
       <c r="E3" s="27" t="n">
         <v>150</v>
       </c>
-      <c r="F3" s="17" t="inlineStr">
-        <is>
-          <t>oui</t>
-        </is>
-      </c>
+      <c r="F3" s="17" t="n"/>
       <c r="G3" s="17" t="inlineStr">
         <is>
           <t>subscription</t>
@@ -7493,7 +7489,11 @@
       <c r="E4" s="29" t="n">
         <v>190</v>
       </c>
-      <c r="F4" s="16" t="n"/>
+      <c r="F4" s="16" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
       <c r="G4" s="16" t="inlineStr">
         <is>
           <t>subscription</t>

</xml_diff>

<commit_message>
Vente flash d'Halloween : -60% jusqu'au 1er novembre
Le meme changement que sur halloween-earn2trade (7f86934), pour que la
branche de brouillon ne reparte pas en arriere : la fenetre Halloween dans
le tableur, la phrase du coupon qui distingue la vente flash du code
permanent, et les prix remises dans le tableau des plans.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/firms/earn2trade.xlsx
+++ b/data/firms/earn2trade.xlsx
@@ -1577,7 +1577,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1976,6 +1976,36 @@
       <c r="F14" t="inlineStr">
         <is>
           <t>not_published</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-10-28T05:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-11-02T04:59:00+00:00</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Halloween · -60%</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>60% off every evaluation and 50% off resets — both apply to your first two months of subscription, purchase date included.</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>60</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>confirmed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Halloween : la carte /compare passe a -60% comme le bandeau
Le meme changement que sur halloween-cartes (f3c4c0b) : la campagne est
renseignee aussi dans l'onglet Offre (`remise_campagne`, `campagne_fin`,
bonus, accroche), que lisent les cartes, les filtres et le tri — l'onglet
Campagnes, lui, ne sert qu'au bandeau et reste cote serveur.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/firms/earn2trade.xlsx
+++ b/data/firms/earn2trade.xlsx
@@ -1512,6 +1512,11 @@
           <t>accroche</t>
         </is>
       </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>60% off every evaluation and 50% off resets — both apply to your first two months of subscription, purchase date included.</t>
+        </is>
+      </c>
       <c r="D10" s="15" t="inlineStr">
         <is>
           <t>Une phrase courte pour le bandeau de campagne du site : ce que l'offre donne, en plus du pourcentage. Vide : le bandeau n'affiche que la remise.</t>
@@ -1524,6 +1529,9 @@
           <t>remise_campagne</t>
         </is>
       </c>
+      <c r="B11" t="n">
+        <v>60</v>
+      </c>
       <c r="D11" s="15" t="inlineStr">
         <is>
           <t>Taux d'une campagne a duree limitee, en %. Il remplace « remise » jusqu'a « campagne_fin », puis la fiche revient a « remise ».</t>
@@ -1536,6 +1544,11 @@
           <t>campagne_fin</t>
         </is>
       </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-11-02T04:59:00+00:00</t>
+        </is>
+      </c>
       <c r="D12" s="15" t="inlineStr">
         <is>
           <t>Fin de la campagne, date et heure ISO. Passee, le taux de campagne et l'accroche disparaissent, l'offre permanente reste.</t>
@@ -1546,6 +1559,11 @@
       <c r="A13" s="15" t="inlineStr">
         <is>
           <t>bonus</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>+50% off resets</t>
         </is>
       </c>
       <c r="D13" s="15" t="inlineStr">

</xml_diff>